<commit_message>
Add frontend screen API contract deck
</commit_message>
<xml_diff>
--- a/html/project-links/MACHINE_IQ_GitHub_산출물_링크_20260828.xlsx
+++ b/html/project-links/MACHINE_IQ_GitHub_산출물_링크_20260828.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub 링크 모음" sheetId="1" r:id="Rf3078575b0d84663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub 링크 모음" sheetId="1" r:id="R534ed25fd9ec4f41"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -768,6 +768,26 @@
         <x:v>현재 문서</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="40" customHeight="1">
+      <x:c r="A24" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>개발 문서</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>프론트 화면별 변수·API 계약</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>https://giry02.github.io/linq/html/developer-atlas/frontend-screen-contracts/</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>https://github.com/giry02/linq/tree/main/html/developer-atlas/frontend-screen-contracts</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>화면별 입력·출력 필드, 타입, 필수·빈값, 향후 API 계약</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Update requirement review battery screens and Figma links
</commit_message>
<xml_diff>
--- a/html/project-links/MACHINE_IQ_GitHub_산출물_링크_20260828.xlsx
+++ b/html/project-links/MACHINE_IQ_GitHub_산출물_링크_20260828.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub 링크 모음" sheetId="1" r:id="R534ed25fd9ec4f41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub 링크 모음" sheetId="1" r:id="Rc5605422680b4138"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -46,7 +46,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -61,6 +61,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9D9D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -103,7 +108,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -136,6 +141,23 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -350,7 +372,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>MACHINE IQ GitHub 산출물 링크 모음</x:v>
+        <x:v>MACHINE IQ 산출물 · Figma 링크 모음</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -360,7 +382,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>기준일: 2026-08-28 · GitHub Pages 공개 주소와 저장소 경로</x:v>
+        <x:v>기준일: 2026-08-28 · GitHub Pages, 저장소, Figma Page 1 경로</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -382,7 +404,7 @@
         <x:v>웹 주소</x:v>
       </x:c>
       <x:c r="E4" s="10" t="str">
-        <x:v>GitHub 폴더/파일</x:v>
+        <x:v>저장소/Figma 경로</x:v>
       </x:c>
       <x:c r="F4" s="10" t="str">
         <x:v>비고</x:v>
@@ -768,24 +790,64 @@
         <x:v>현재 문서</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="40" customHeight="1">
-      <x:c r="A24" t="n">
+    <x:row r="24" ht="44" customHeight="1">
+      <x:c r="A24" s="25" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B24" t="str">
+      <x:c r="B24" s="25" t="str">
         <x:v>개발 문서</x:v>
       </x:c>
-      <x:c r="C24" t="str">
+      <x:c r="C24" s="24" t="str">
         <x:v>프론트 화면별 변수·API 계약</x:v>
       </x:c>
-      <x:c r="D24" t="str">
+      <x:c r="D24" s="24" t="str">
         <x:v>https://giry02.github.io/linq/html/developer-atlas/frontend-screen-contracts/</x:v>
       </x:c>
-      <x:c r="E24" t="str">
+      <x:c r="E24" s="24" t="str">
         <x:v>https://github.com/giry02/linq/tree/main/html/developer-atlas/frontend-screen-contracts</x:v>
       </x:c>
-      <x:c r="F24" t="str">
+      <x:c r="F24" s="24" t="str">
         <x:v>화면별 입력·출력 필드, 타입, 필수·빈값, 향후 API 계약</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="44" customHeight="1">
+      <x:c r="A25" s="25" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B25" s="25" t="str">
+        <x:v>Figma</x:v>
+      </x:c>
+      <x:c r="C25" s="24" t="str">
+        <x:v>LIN-Q Page 1 원본</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>https://www.figma.com/design/djG9ZrdP7sNzK78rMAfQ3U/LIN-Q?node-id=1-3</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>https://www.figma.com/design/djG9ZrdP7sNzK78rMAfQ3U/LIN-Q?node-id=1-3&amp;p=f</x:v>
+      </x:c>
+      <x:c r="F25" s="24" t="str">
+        <x:v>사용 기준 Page 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="44" customHeight="1">
+      <x:c r="A26" s="25" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B26" s="25" t="str">
+        <x:v>Figma</x:v>
+      </x:c>
+      <x:c r="C26" s="24" t="str">
+        <x:v>Page 1 플릿·딜러 화면 위치</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>https://www.figma.com/design/djG9ZrdP7sNzK78rMAfQ3U/LIN-Q?node-id=1-8</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>https://www.figma.com/design/djG9ZrdP7sNzK78rMAfQ3U/LIN-Q?node-id=1-8&amp;p=f</x:v>
+      </x:c>
+      <x:c r="F26" s="24" t="str">
+        <x:v>좌측 플릿 · 우측 딜러</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>